<commit_message>
changer apparance et alertes
</commit_message>
<xml_diff>
--- a/reports/rapport-tests.xlsx
+++ b/reports/rapport-tests.xlsx
@@ -1,19 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09C351F2-B92E-425C-B320-C7581DDB0D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Hôtels" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Chambres" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Pensions" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Destination" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Example" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Hotel" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Reservation" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Voyage" state="visible" r:id="rId11"/>
+    <sheet name="Hôtels" sheetId="1" r:id="rId1"/>
+    <sheet name="Chambres" sheetId="2" r:id="rId2"/>
+    <sheet name="Pensions" sheetId="3" r:id="rId3"/>
+    <sheet name="Destination" sheetId="4" r:id="rId4"/>
+    <sheet name="Example" sheetId="5" r:id="rId5"/>
+    <sheet name="Hotel" sheetId="6" r:id="rId6"/>
+    <sheet name="Reservation" sheetId="7" r:id="rId7"/>
+    <sheet name="Voyage" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -449,18 +454,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="4">
@@ -835,14 +842,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="6" width="18" customWidth="1"/>
+    <col min="1" max="1" width="2.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="116.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -862,7 +874,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -882,7 +894,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -902,7 +914,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -922,7 +934,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -942,7 +954,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -964,19 +976,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G50"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="7" width="18" customWidth="1"/>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -999,7 +1017,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1022,7 +1040,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1045,7 +1063,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1068,7 +1086,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1091,7 +1109,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1114,7 +1132,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1137,7 +1155,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1160,7 +1178,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1183,7 +1201,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1206,7 +1224,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1229,7 +1247,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1252,7 +1270,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1275,7 +1293,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1298,7 +1316,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1321,7 +1339,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1344,7 +1362,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1367,7 +1385,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1390,7 +1408,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1413,7 +1431,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1436,7 +1454,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1459,7 +1477,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1482,7 +1500,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1505,7 +1523,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1528,7 +1546,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1551,7 +1569,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1574,7 +1592,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1597,7 +1615,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1620,7 +1638,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1643,7 +1661,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1666,7 +1684,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1689,7 +1707,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1712,7 +1730,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1735,7 +1753,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1758,7 +1776,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1781,7 +1799,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1804,7 +1822,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1827,7 +1845,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1850,7 +1868,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1873,7 +1891,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1896,7 +1914,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1919,7 +1937,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1942,7 +1960,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1965,7 +1983,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1988,7 +2006,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2011,7 +2029,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2034,7 +2052,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2057,7 +2075,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2080,7 +2098,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2103,7 +2121,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2128,19 +2146,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G196"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="7" width="18" customWidth="1"/>
+    <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2163,7 +2187,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2186,7 +2210,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2209,7 +2233,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2232,7 +2256,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2255,7 +2279,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2278,7 +2302,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2301,7 +2325,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2324,7 +2348,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2347,7 +2371,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2370,7 +2394,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2393,7 +2417,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2416,7 +2440,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2439,7 +2463,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2462,7 +2486,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2485,7 +2509,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2508,7 +2532,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2531,7 +2555,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2554,7 +2578,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2577,7 +2601,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2600,7 +2624,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2623,7 +2647,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2646,7 +2670,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2669,7 +2693,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2692,7 +2716,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2715,7 +2739,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2738,7 +2762,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2761,7 +2785,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2784,7 +2808,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2807,7 +2831,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2830,7 +2854,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2853,7 +2877,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2876,7 +2900,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2899,7 +2923,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2922,7 +2946,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2945,7 +2969,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2968,7 +2992,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2991,7 +3015,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3014,7 +3038,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3037,7 +3061,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3060,7 +3084,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3083,7 +3107,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3106,7 +3130,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3129,7 +3153,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -3152,7 +3176,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -3175,7 +3199,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -3198,7 +3222,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -3221,7 +3245,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -3244,7 +3268,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -3267,7 +3291,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -3290,7 +3314,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -3313,7 +3337,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -3336,7 +3360,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -3359,7 +3383,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -3382,7 +3406,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -3405,7 +3429,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -3428,7 +3452,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -3451,7 +3475,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -3474,7 +3498,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -3497,7 +3521,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -3520,7 +3544,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -3543,7 +3567,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -3566,7 +3590,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -3589,7 +3613,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -3612,7 +3636,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -3635,7 +3659,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -3658,7 +3682,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -3681,7 +3705,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -3704,7 +3728,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -3727,7 +3751,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -3750,7 +3774,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -3773,7 +3797,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -3796,7 +3820,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -3819,7 +3843,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -3842,7 +3866,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>74</v>
       </c>
@@ -3865,7 +3889,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>75</v>
       </c>
@@ -3888,7 +3912,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>76</v>
       </c>
@@ -3911,7 +3935,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>77</v>
       </c>
@@ -3934,7 +3958,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>78</v>
       </c>
@@ -3957,7 +3981,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>79</v>
       </c>
@@ -3980,7 +4004,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>80</v>
       </c>
@@ -4003,7 +4027,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>81</v>
       </c>
@@ -4026,7 +4050,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>82</v>
       </c>
@@ -4049,7 +4073,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>83</v>
       </c>
@@ -4072,7 +4096,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>84</v>
       </c>
@@ -4095,7 +4119,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>85</v>
       </c>
@@ -4118,7 +4142,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>86</v>
       </c>
@@ -4141,7 +4165,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>87</v>
       </c>
@@ -4164,7 +4188,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>88</v>
       </c>
@@ -4187,7 +4211,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>89</v>
       </c>
@@ -4210,7 +4234,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>90</v>
       </c>
@@ -4233,7 +4257,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>91</v>
       </c>
@@ -4256,7 +4280,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>92</v>
       </c>
@@ -4279,7 +4303,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>93</v>
       </c>
@@ -4302,7 +4326,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>94</v>
       </c>
@@ -4325,7 +4349,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>95</v>
       </c>
@@ -4348,7 +4372,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>96</v>
       </c>
@@ -4371,7 +4395,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>97</v>
       </c>
@@ -4394,7 +4418,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>98</v>
       </c>
@@ -4417,7 +4441,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>99</v>
       </c>
@@ -4440,7 +4464,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>100</v>
       </c>
@@ -4463,7 +4487,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>101</v>
       </c>
@@ -4486,7 +4510,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>102</v>
       </c>
@@ -4509,7 +4533,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>103</v>
       </c>
@@ -4532,7 +4556,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>104</v>
       </c>
@@ -4555,7 +4579,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>105</v>
       </c>
@@ -4578,7 +4602,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>106</v>
       </c>
@@ -4601,7 +4625,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>107</v>
       </c>
@@ -4624,7 +4648,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>108</v>
       </c>
@@ -4647,7 +4671,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>109</v>
       </c>
@@ -4670,7 +4694,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>110</v>
       </c>
@@ -4693,7 +4717,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>111</v>
       </c>
@@ -4716,7 +4740,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>112</v>
       </c>
@@ -4739,7 +4763,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>113</v>
       </c>
@@ -4762,7 +4786,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>114</v>
       </c>
@@ -4785,7 +4809,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>115</v>
       </c>
@@ -4808,7 +4832,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>116</v>
       </c>
@@ -4831,7 +4855,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>117</v>
       </c>
@@ -4854,7 +4878,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>118</v>
       </c>
@@ -4877,7 +4901,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>119</v>
       </c>
@@ -4900,7 +4924,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>120</v>
       </c>
@@ -4923,7 +4947,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>121</v>
       </c>
@@ -4946,7 +4970,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>122</v>
       </c>
@@ -4969,7 +4993,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>123</v>
       </c>
@@ -4992,7 +5016,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>124</v>
       </c>
@@ -5015,7 +5039,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>125</v>
       </c>
@@ -5038,7 +5062,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>126</v>
       </c>
@@ -5061,7 +5085,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>127</v>
       </c>
@@ -5084,7 +5108,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>128</v>
       </c>
@@ -5107,7 +5131,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>129</v>
       </c>
@@ -5130,7 +5154,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>130</v>
       </c>
@@ -5153,7 +5177,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>131</v>
       </c>
@@ -5176,7 +5200,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>132</v>
       </c>
@@ -5199,7 +5223,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>133</v>
       </c>
@@ -5222,7 +5246,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>134</v>
       </c>
@@ -5245,7 +5269,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>135</v>
       </c>
@@ -5268,7 +5292,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>136</v>
       </c>
@@ -5291,7 +5315,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>137</v>
       </c>
@@ -5314,7 +5338,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>138</v>
       </c>
@@ -5337,7 +5361,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>139</v>
       </c>
@@ -5360,7 +5384,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>140</v>
       </c>
@@ -5383,7 +5407,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>141</v>
       </c>
@@ -5406,7 +5430,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>142</v>
       </c>
@@ -5429,7 +5453,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>143</v>
       </c>
@@ -5452,7 +5476,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>144</v>
       </c>
@@ -5475,7 +5499,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>145</v>
       </c>
@@ -5498,7 +5522,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>146</v>
       </c>
@@ -5521,7 +5545,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>147</v>
       </c>
@@ -5544,7 +5568,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>148</v>
       </c>
@@ -5567,7 +5591,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>149</v>
       </c>
@@ -5590,7 +5614,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>150</v>
       </c>
@@ -5613,7 +5637,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>151</v>
       </c>
@@ -5636,7 +5660,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>152</v>
       </c>
@@ -5659,7 +5683,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>153</v>
       </c>
@@ -5682,7 +5706,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>154</v>
       </c>
@@ -5705,7 +5729,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>155</v>
       </c>
@@ -5728,7 +5752,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>156</v>
       </c>
@@ -5751,7 +5775,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>157</v>
       </c>
@@ -5774,7 +5798,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>158</v>
       </c>
@@ -5797,7 +5821,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>159</v>
       </c>
@@ -5820,7 +5844,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>160</v>
       </c>
@@ -5843,7 +5867,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>161</v>
       </c>
@@ -5866,7 +5890,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>162</v>
       </c>
@@ -5889,7 +5913,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>163</v>
       </c>
@@ -5912,7 +5936,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>164</v>
       </c>
@@ -5935,7 +5959,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>165</v>
       </c>
@@ -5958,7 +5982,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>166</v>
       </c>
@@ -5981,7 +6005,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>167</v>
       </c>
@@ -6004,7 +6028,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>168</v>
       </c>
@@ -6027,7 +6051,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>169</v>
       </c>
@@ -6050,7 +6074,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>170</v>
       </c>
@@ -6073,7 +6097,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>171</v>
       </c>
@@ -6096,7 +6120,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>172</v>
       </c>
@@ -6119,7 +6143,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>173</v>
       </c>
@@ -6142,7 +6166,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>174</v>
       </c>
@@ -6165,7 +6189,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>175</v>
       </c>
@@ -6188,7 +6212,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>176</v>
       </c>
@@ -6211,7 +6235,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>177</v>
       </c>
@@ -6234,7 +6258,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>178</v>
       </c>
@@ -6257,7 +6281,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>179</v>
       </c>
@@ -6280,7 +6304,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>180</v>
       </c>
@@ -6303,7 +6327,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>181</v>
       </c>
@@ -6326,7 +6350,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>182</v>
       </c>
@@ -6349,7 +6373,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>183</v>
       </c>
@@ -6372,7 +6396,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>184</v>
       </c>
@@ -6395,7 +6419,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>185</v>
       </c>
@@ -6418,7 +6442,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>186</v>
       </c>
@@ -6441,7 +6465,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>187</v>
       </c>
@@ -6464,7 +6488,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>188</v>
       </c>
@@ -6487,7 +6511,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>189</v>
       </c>
@@ -6510,7 +6534,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>190</v>
       </c>
@@ -6533,7 +6557,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>191</v>
       </c>
@@ -6556,7 +6580,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>192</v>
       </c>
@@ -6579,7 +6603,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>193</v>
       </c>
@@ -6602,7 +6626,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>194</v>
       </c>
@@ -6625,7 +6649,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>195</v>
       </c>
@@ -6650,19 +6674,26 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="8" width="18" customWidth="1"/>
+    <col min="1" max="1" width="2.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6688,7 +6719,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -6708,13 +6739,13 @@
         <v>56</v>
       </c>
       <c r="G2">
-        <v>0.028516</v>
+        <v>2.8516E-2</v>
       </c>
       <c r="H2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -6734,13 +6765,13 @@
         <v>56</v>
       </c>
       <c r="G3">
-        <v>0.000488</v>
+        <v>4.8799999999999999E-4</v>
       </c>
       <c r="H3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -6760,13 +6791,13 @@
         <v>56</v>
       </c>
       <c r="G4">
-        <v>0.000223</v>
+        <v>2.23E-4</v>
       </c>
       <c r="H4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -6786,13 +6817,13 @@
         <v>56</v>
       </c>
       <c r="G5">
-        <v>0.000181</v>
+        <v>1.8100000000000001E-4</v>
       </c>
       <c r="H5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -6812,13 +6843,13 @@
         <v>56</v>
       </c>
       <c r="G6">
-        <v>0.000128</v>
+        <v>1.2799999999999999E-4</v>
       </c>
       <c r="H6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -6838,7 +6869,7 @@
         <v>56</v>
       </c>
       <c r="G7">
-        <v>0.000667</v>
+        <v>6.6699999999999995E-4</v>
       </c>
       <c r="H7" t="s">
         <v>57</v>
@@ -6846,19 +6877,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="6" width="18" customWidth="1"/>
+    <col min="1" max="1" width="2.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6878,7 +6914,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -6892,7 +6928,7 @@
         <v>56</v>
       </c>
       <c r="E2">
-        <v>0.000131</v>
+        <v>1.3100000000000001E-4</v>
       </c>
       <c r="F2" t="s">
         <v>57</v>
@@ -6900,19 +6936,27 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="9" width="18" customWidth="1"/>
+    <col min="1" max="1" width="2.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6941,7 +6985,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -6964,13 +7008,13 @@
         <v>56</v>
       </c>
       <c r="H2">
-        <v>0.000799</v>
+        <v>7.9900000000000001E-4</v>
       </c>
       <c r="I2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -6993,13 +7037,13 @@
         <v>56</v>
       </c>
       <c r="H3">
-        <v>0.000151</v>
+        <v>1.5100000000000001E-4</v>
       </c>
       <c r="I3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -7022,13 +7066,13 @@
         <v>56</v>
       </c>
       <c r="H4">
-        <v>0.000234</v>
+        <v>2.34E-4</v>
       </c>
       <c r="I4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -7051,13 +7095,13 @@
         <v>56</v>
       </c>
       <c r="H5">
-        <v>0.000119</v>
+        <v>1.1900000000000001E-4</v>
       </c>
       <c r="I5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -7080,13 +7124,13 @@
         <v>56</v>
       </c>
       <c r="H6">
-        <v>0.000119</v>
+        <v>1.1900000000000001E-4</v>
       </c>
       <c r="I6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -7109,13 +7153,13 @@
         <v>56</v>
       </c>
       <c r="H7">
-        <v>0.000141</v>
+        <v>1.4100000000000001E-4</v>
       </c>
       <c r="I7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -7138,13 +7182,13 @@
         <v>56</v>
       </c>
       <c r="H8">
-        <v>0.000122</v>
+        <v>1.22E-4</v>
       </c>
       <c r="I8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -7167,7 +7211,7 @@
         <v>56</v>
       </c>
       <c r="H9">
-        <v>0.000114</v>
+        <v>1.1400000000000001E-4</v>
       </c>
       <c r="I9" t="s">
         <v>57</v>
@@ -7175,19 +7219,29 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K18"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="11" width="18" customWidth="1"/>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7222,7 +7276,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -7251,13 +7305,13 @@
         <v>56</v>
       </c>
       <c r="J2">
-        <v>0.000778</v>
+        <v>7.7800000000000005E-4</v>
       </c>
       <c r="K2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -7286,13 +7340,13 @@
         <v>56</v>
       </c>
       <c r="J3">
-        <v>0.000167</v>
+        <v>1.6699999999999999E-4</v>
       </c>
       <c r="K3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -7321,13 +7375,13 @@
         <v>56</v>
       </c>
       <c r="J4">
-        <v>0.000166</v>
+        <v>1.66E-4</v>
       </c>
       <c r="K4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -7356,13 +7410,13 @@
         <v>56</v>
       </c>
       <c r="J5">
-        <v>0.000145</v>
+        <v>1.45E-4</v>
       </c>
       <c r="K5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -7391,13 +7445,13 @@
         <v>56</v>
       </c>
       <c r="J6">
-        <v>0.000644</v>
+        <v>6.4400000000000004E-4</v>
       </c>
       <c r="K6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -7426,13 +7480,13 @@
         <v>56</v>
       </c>
       <c r="J7">
-        <v>0.000224</v>
+        <v>2.24E-4</v>
       </c>
       <c r="K7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -7461,13 +7515,13 @@
         <v>56</v>
       </c>
       <c r="J8">
-        <v>0.000169</v>
+        <v>1.6899999999999999E-4</v>
       </c>
       <c r="K8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -7496,13 +7550,13 @@
         <v>56</v>
       </c>
       <c r="J9">
-        <v>0.000174</v>
+        <v>1.74E-4</v>
       </c>
       <c r="K9" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -7531,13 +7585,13 @@
         <v>56</v>
       </c>
       <c r="J10">
-        <v>0.00014</v>
+        <v>1.3999999999999999E-4</v>
       </c>
       <c r="K10" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -7566,13 +7620,13 @@
         <v>56</v>
       </c>
       <c r="J11">
-        <v>0.000112</v>
+        <v>1.12E-4</v>
       </c>
       <c r="K11" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -7601,13 +7655,13 @@
         <v>56</v>
       </c>
       <c r="J12">
-        <v>0.000121</v>
+        <v>1.21E-4</v>
       </c>
       <c r="K12" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -7636,13 +7690,13 @@
         <v>56</v>
       </c>
       <c r="J13">
-        <v>0.000132</v>
+        <v>1.3200000000000001E-4</v>
       </c>
       <c r="K13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -7671,13 +7725,13 @@
         <v>56</v>
       </c>
       <c r="J14">
-        <v>0.000136</v>
+        <v>1.36E-4</v>
       </c>
       <c r="K14" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -7706,13 +7760,13 @@
         <v>56</v>
       </c>
       <c r="J15">
-        <v>0.000117</v>
+        <v>1.17E-4</v>
       </c>
       <c r="K15" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -7741,13 +7795,13 @@
         <v>56</v>
       </c>
       <c r="J16">
-        <v>0.000132</v>
+        <v>1.3200000000000001E-4</v>
       </c>
       <c r="K16" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -7776,13 +7830,13 @@
         <v>56</v>
       </c>
       <c r="J17">
-        <v>0.000108</v>
+        <v>1.08E-4</v>
       </c>
       <c r="K17" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -7811,7 +7865,7 @@
         <v>56</v>
       </c>
       <c r="J18">
-        <v>0.00161</v>
+        <v>1.6100000000000001E-3</v>
       </c>
       <c r="K18" t="s">
         <v>57</v>
@@ -7819,19 +7873,26 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="8" width="18" customWidth="1"/>
+    <col min="1" max="1" width="2.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7857,7 +7918,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -7877,13 +7938,13 @@
         <v>56</v>
       </c>
       <c r="G2">
-        <v>0.000593</v>
+        <v>5.9299999999999999E-4</v>
       </c>
       <c r="H2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -7903,13 +7964,13 @@
         <v>56</v>
       </c>
       <c r="G3">
-        <v>0.000155</v>
+        <v>1.55E-4</v>
       </c>
       <c r="H3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -7929,13 +7990,13 @@
         <v>56</v>
       </c>
       <c r="G4">
-        <v>0.000123</v>
+        <v>1.2300000000000001E-4</v>
       </c>
       <c r="H4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -7955,13 +8016,13 @@
         <v>56</v>
       </c>
       <c r="G5">
-        <v>0.000131</v>
+        <v>1.3100000000000001E-4</v>
       </c>
       <c r="H5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -7981,13 +8042,13 @@
         <v>56</v>
       </c>
       <c r="G6">
-        <v>0.000116</v>
+        <v>1.16E-4</v>
       </c>
       <c r="H6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -8007,13 +8068,13 @@
         <v>56</v>
       </c>
       <c r="G7">
-        <v>0.000114</v>
+        <v>1.1400000000000001E-4</v>
       </c>
       <c r="H7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -8033,13 +8094,13 @@
         <v>56</v>
       </c>
       <c r="G8">
-        <v>0.00012</v>
+        <v>1.2E-4</v>
       </c>
       <c r="H8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -8059,7 +8120,7 @@
         <v>56</v>
       </c>
       <c r="G9">
-        <v>0.000117</v>
+        <v>1.17E-4</v>
       </c>
       <c r="H9" t="s">
         <v>57</v>
@@ -8067,6 +8128,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>